<commit_message>
Plan coverage expansion for downloader scripts tests
Agent-Logs-Url: https://github.com/matheus-rech/ICSKG/sessions/d9630e31-7ae3-4e80-9a84-42f84e0ba6e2

Co-authored-by: matheus-rech <71096630+matheus-rech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/ifgf_sample.xlsx
+++ b/tests/fixtures/ifgf_sample.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
feat: improve pipeline extractors, add regression results, rewrite CLAUDE.md
Refactor IFGF, CNES, IDHM, and census sanitation extractors for robustness.
Enhance assemble_panel and utils with better error handling. Add dose-response,
Hausman test, regression tables, sensitivity analysis, and spatial results.
Rewrite CLAUDE.md with concise project docs and domain context.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/ifgf_sample.xlsx
+++ b/tests/fixtures/ifgf_sample.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>